<commit_message>
JBoss EAP 8.1 前提で server.log 問題を再検討
- EAP 8.1 → WildFly 35 → WildFly Core 27 → jboss-logmanager 2.1.19.Final /
  wildfly-common 1.7.0.Final を上流 POM で特定し、同じ依存で再現を再実行
  （初版の「EAP 8 は logmanager 3.x 系」の記述を訂正）
- EAP 8 の仕様変更（コンテナが読むのは logging.properties / jboss-logging.properties
  だけ、log4j 1.x 提供廃止）に基づき原因候補1b（アプリ同梱 reload4j 等）を追加し、
  reload4j 1.2.26 と JBoss FILE の共存を MixedLibraryRepro.java で再現
- audit-logging-config.sh：デプロイメント内設定を「誰が読むか」で分類し、
  同梱 jar と jboss-deployment-structure.xml の除外から有効性を判定
- 対策 J2 を J2a（use-deployment-logging-config）と J2b（アプリ側で出力先変更）に分割
- md 第16章と Excel 14〜19・00 シートを EAP 8.1 前提に改訂

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UmEw33mt5tCcgER5mYeATG
</commit_message>
<xml_diff>
--- a/Log4j2_EFS_ローリングアップデート_FD競合_解説.xlsx
+++ b/Log4j2_EFS_ローリングアップデート_FD競合_解説.xlsx
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1372,7 +1372,7 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>■ 追加検討（2026-09-24）：JBoss EAP の server.log が前日付ファイルに追記され続ける問題</t>
+          <t>■ 追加検討（2026-09-24／EAP 8.1 前提）：JBoss EAP 8.1 の server.log が前日付ファイルに追記され続ける問題</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>タスクIDディレクトリでは防げない。犯人は同じタスクの内側（2つ目のハンドラ・stdout リダイレクト）か外部の rename</t>
+          <t>タスクIDディレクトリでは防げない。犯人は同じタスクの内側（2つ目のハンドラ・同梱 reload4j 等・stdout リダイレクト）か外部の rename</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr"/>
@@ -1456,53 +1456,79 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="51" customHeight="1">
-      <c r="A35" s="5" t="n">
+    <row r="35" ht="96" customHeight="1">
+      <c r="A35" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>実物の jboss-logmanager で再現済み。原因候補1・3a は症状と完全一致し、前日分のログが毎日消える</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr"/>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Files.move(REPLACE_EXISTING) で前日分を上書き削除。翌日も繰り返し、日付名が1日ずれる</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>server.log.&lt;日付&gt; の先頭行の日付を確認</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>16, 17</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="81" customHeight="1">
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>EAP 8.1 固有：コンテナは log4j 1.x を提供しないため、アプリ同梱の reload4j が log4j.xml を読んで server.log を開き rename する。use-deployment-logging-config では止まらない</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr"/>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>WildFly Core 27 のソース（コンテナが読むのは logging.properties／jboss-logging.properties だけ）と reload4j 1.2.26 での再現</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>アプリ側で出力先を server.log 以外へ（J2b）</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>14, 15, 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="66" customHeight="1">
       <c r="A36" s="5" t="n">
         <v>4</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>対応：FILE 以外のハンドラを外す／デプロイメント内ログ設定を無効化／リダイレクトしない／logrotate に触らせない／TZ=JST。恒久策は JSON で stdout</t>
+          <t>EAP 8.1 と同じ jboss-logmanager 2.1.19.Final で再現済み。原因候補1・1b・3a は症状と完全一致し、前日分のログが毎日消える</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr"/>
       <c r="D36" s="6" t="inlineStr">
         <is>
+          <t>Files.move(REPLACE_EXISTING) で前日分を上書き削除。翌日も繰り返し、日付名が1日ずれる</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>server.log.&lt;日付&gt; の先頭行の日付を確認</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>16, 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="96" customHeight="1">
+      <c r="A37" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>対応：FILE 以外のハンドラを外す／logging.properties 系を無効化／同梱ライブラリの出力先を変更／リダイレクトしない／logrotate に触らせない／TZ=JST。恒久策は JSON で stdout</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
           <t>jboss/cli・jboss/bin に実装</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>J1〜J8</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -4385,7 +4411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4398,7 +4424,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【追記 2026-09-24】JBoss EAP の server.log が「前日付ファイル」に追記され続ける問題 — 結論</t>
+          <t>【追記 2026-09-24／EAP 8.1 前提で再検討】JBoss EAP 8.1 の server.log が「前日付ファイル」に追記され続ける問題 — 結論</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4494,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="111" customHeight="1">
+    <row r="7" ht="156" customHeight="1">
       <c r="A7" s="9" t="n">
         <v>2</v>
       </c>
@@ -4479,7 +4505,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>(1) 同じ JVM 内で server.log を開く2つ目のハンドラ（別名ハンドラ・logging-profile・WAR 同梱の logging.properties / log4j.xml / log4j2.xml）、(2) entrypoint の stdout リダイレクト、(3) logrotate・収集バッチ・別ホストの cron による rename。いずれも同じディレクトリの中で起きる。</t>
+          <t>(1) 同じ JVM 内で server.log を開く2つ目のハンドラ（別名ハンドラ・logging-profile・WAR 同梱の logging.properties / jboss-logging.properties）、(1b) アプリが同梱した reload4j 等のアペンダ（EAP 8 はコンテナが log4j 1.x を提供しないため、log4j.xml はアプリのライブラリ自身が読む）、(2) entrypoint の stdout リダイレクト、(3) logrotate・収集バッチ・別ホストの cron による rename。いずれも同じディレクトリの中で起きる。</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -4493,7 +4519,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="96" customHeight="1">
+    <row r="8" ht="126" customHeight="1">
       <c r="A8" s="5" t="n">
         <v>3</v>
       </c>
@@ -4504,7 +4530,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>2つ目のハンドラを app.log へ向け直す／use-deployment-logging-config=false、stdout を server.log へリダイレクトしない、logrotate 等に server.log を触らせない。TZ=Asia/Tokyo も設定。恒久策は server.log をやめて JSON で stdout → FireLens/awslogs。</t>
+          <t>2つ目のハンドラを app.log へ向け直す／use-deployment-logging-config=false（logging.properties 系だけに効く）、同梱 reload4j 等はアプリ側で出力先を変更、stdout を server.log へリダイレクトしない、logrotate 等に server.log を触らせない。TZ=Asia/Tokyo も設定。恒久策は server.log をやめて JSON で stdout → FireLens/awslogs。</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -4524,7 +4550,7 @@
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>実物の jboss-logmanager（2.1.19.Final ＝ EAP 7.4 系）で再現済み。原因候補1と3a が症状と完全一致し、どちらも前日分のログが消える</t>
+          <t>EAP 8.1 と同じ jboss-logmanager 2.1.19.Final で再現済み。原因候補1・1b・3a が症状と完全一致し、いずれも前日分のログが消える</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -4546,92 +4572,92 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>■ 推理の出発点（推測ではなく、仕組みから必ずそうなること）</t>
+          <t>■ 前提バージョン（JBoss EAP 8.1）— 2026-09-24 に Maven Central の上流 POM で確認</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>STEP</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>事実</t>
+          <t>層</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>説明</t>
+          <t>バージョン</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>ここから言えること</t>
+          <t>根拠</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
     </row>
-    <row r="13" ht="66" customHeight="1">
+    <row r="13" ht="21" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>JBoss が開くのは常に server.log</t>
+          <t>JBoss EAP</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>rollOver() は setFileInternal(null) で自分の FD を閉じ、server.log を日付名へ move し、setFileInternal(file) で server.log を開き直す。</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>日付名で開く人はいない</t>
+          <t>対象</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="21" customHeight="1">
       <c r="A14" s="5" t="n">
         <v>2</v>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>それでも日付ファイルに今日のログが増えている</t>
+          <t>上流の WildFly</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>ls -l で server.log.2026-09-18 のサイズと mtime が増え続けている</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>誰かが書いている</t>
+          <t>EAP 8.1 は WildFly 35 ベース</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
     </row>
-    <row r="15" ht="51" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>日付名で開いた人はいないので、書けるのは「server.log だった頃に開いた FD」だけ</t>
+          <t>WildFly Core</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>rename は FD に影響しない（第3章 3.2）</t>
+          <t>27.0.x</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>古い FD を持ち続けている書き手がいる</t>
+          <t>wildfly-parent-35.0.0.Final.pom の version.org.wildfly.core</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr"/>
@@ -4642,426 +4668,727 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
+          <t>jboss-logmanager</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>2.1.19.Final</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>wildfly-core-parent-27.0.x.pom の version.org.jboss.logmanager.jboss-logmanager。製品版は -redhat-NNNNN 付き</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>wildfly-common</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>1.7.0.Final</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>同上の version.org.wildfly.common</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>※ 実機では ls $JBOSS_HOME/modules/system/layers/base/org/jboss/logmanager/main/ で確認。初版で「EAP 8 は 3.x 系」と記載したのは誤りで、EAP 8.1 は 2.1 系。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>■ EAP 8（8.0 以降）で変わった、今回の原因に直結する仕様（WildFly Core 27 のソースで確認）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>仕様</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>EAP 8.1 での挙動</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>今回への影響</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="51" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>コンテナが読むデプロイメント内ログ設定</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>META-INF または WEB-INF/classes の logging.properties と jboss-logging.properties だけ</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>use-deployment-logging-config=false で止められるのはこの2つだけ</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="66" customHeight="1">
+      <c r="A23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>log4j 1.x</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>コンテナが提供しなくなった。log4j.xml / log4j.properties / jboss-log4j.xml をコンテナは読まない</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>旧アプリは reload4j 等を WAR に同梱して動かす。reload4j 自身が log4j.xml を読み、自分で server.log を開いて rename する。コンテナの設定では止まらない（原因候補1b）</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24" ht="51" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Log4j2 API</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>コンテナが org.apache.logging.log4j.api を自動追加し JBoss LogManager に流す</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>アプリの log4j2.xml は通常使われない。log4j-core 同梱かつ API モジュール除外のときだけ log4j-core 自身がファイルを開く</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>SLF4J</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>コンテナが org.slf4j を追加</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>logback.xml も logback 同梱かつ slf4j モジュール除外のときだけ有効</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="66" customHeight="1">
+      <c r="A26" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>起動時ログ</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>standalone.sh が -Dorg.jboss.boot.log.file=$JBOSS_LOG_DIR/server.log を渡し、logging.properties の FILE が起動直後から書く</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>subsystem の FILE と同名で引き継がれる同じハンドラなので2人目にはならない。JBOSS_LOG_DIR と jboss.server.log.dir が違うと起動直後だけ別の場所に書かれる（J6）</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="51" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>インストールマネージャ</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>JVM が終了コード 20 で終わると standalone.sh が installation-manager.sh を起動し server.log に書かせる</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>JVM 終了後に順番に書くだけ。原因ではない</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>■ 推理の出発点（推測ではなく、仕組みから必ずそうなること）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>STEP</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>事実</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>ここから言えること</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31" ht="66" customHeight="1">
+      <c r="A31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>JBoss が開くのは常に server.log</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>rollOver() は setFileInternal(null) で自分の FD を閉じ、server.log を日付名へ move し、setFileInternal(file) で server.log を開き直す。</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>日付名で開く人はいない</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>それでも日付ファイルに今日のログが増えている</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>ls -l で server.log.2026-09-18 のサイズと mtime が増え続けている</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>誰かが書いている</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33" ht="51" customHeight="1">
+      <c r="A33" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>日付名で開いた人はいないので、書けるのは「server.log だった頃に開いた FD」だけ</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>rename は FD に影響しない（第3章 3.2）</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>古い FD を持ち続けている書き手がいる</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34" ht="51" customHeight="1">
+      <c r="A34" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
           <t>FILE ハンドラは回転時に自分の FD を必ず開き直す</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>→ 古い FD の持ち主は「FILE 以外の書き手」か、「FILE の回転後に別の誰かがもう一度 rename した」のどちらか</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>JBoss の回転が壊れているのではなく、server.log に FILE 以外の「開く人」か「rename する人」がいる</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>■ タスクIDディレクトリが防ぐもの／防げないもの</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>場面</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>具体例</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>タスクIDディレクトリで防げるか</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>該当</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="42" t="n">
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="44" t="inlineStr">
+      <c r="B38" s="44" t="inlineStr">
         <is>
           <t>別タスクが同じファイルを開く</t>
         </is>
       </c>
-      <c r="C20" s="44" t="inlineStr">
+      <c r="C38" s="44" t="inlineStr">
         <is>
           <t>ローリングアップデート中の旧タスクと新タスク（別ホスト＝別 NFS クライアント）</t>
         </is>
       </c>
-      <c r="D20" s="44" t="inlineStr">
+      <c r="D38" s="44" t="inlineStr">
         <is>
           <t>防げる（パスが違うので同じ inode を開けない）</t>
         </is>
       </c>
-      <c r="E20" s="44" t="inlineStr">
+      <c r="E38" s="44" t="inlineStr">
         <is>
           <t>アプリログ</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="9" t="n">
+    <row r="39" ht="51" customHeight="1">
+      <c r="A39" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>同じ JVM の中の2つの部品が同じ server.log を開く</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>FILE と、CLI で追加した APP_FILE／logging-profile のハンドラ／WAR 同梱の log4j.xml</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>FILE と、CLI で追加した APP_FILE／logging-profile のハンドラ／WAR 同梱の logging.properties／同梱 reload4j の log4j.xml</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
         <is>
           <t>防げない（同じディレクトリの中）</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>原因候補1</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="9" t="n">
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>原因候補1・1b</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>同じコンテナの中でシェルと JVM が同じ server.log を開く</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>entrypoint の standalone.sh &gt;&gt; server.log 2&gt;&amp;1、| tee -a server.log</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D40" s="10" t="inlineStr">
         <is>
           <t>防げない（同じディレクトリの中）</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>原因候補2</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="9" t="n">
+    <row r="41" ht="36" customHeight="1">
+      <c r="A41" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>外部が server.log を名指しで rename する</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>logrotate、収集用 EC2 の cron、S3 退避バッチ、運用手順の mv</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D41" s="10" t="inlineStr">
         <is>
           <t>防げない（パスを知っていれば入ってこられる）</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>原因候補3</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>■ アプリログ（Log4j2）と server.log（JBoss）の比較</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>観点</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>アプリログ（Log4j2 RollingFileAppender）</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>server.log（jboss-logmanager PeriodicRotatingFileHandler）</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>違い</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="5" t="n">
+    <row r="45" ht="36" customHeight="1">
+      <c r="A45" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>回転のきっかけ</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>時刻を過ぎて最初のログイベント</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>時刻を過ぎて最初のログレコード（タイマーは無い）</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>同じ</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="5" t="n">
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>回転の手順</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>close → rename → create</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>close → Files.move(REPLACE_EXISTING) → create</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>同じ</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="21" customHeight="1">
-      <c r="A29" s="5" t="n">
+    <row r="47" ht="21" customHeight="1">
+      <c r="A47" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>回転先が既にあるとき</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>黙って上書き</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>黙って上書き</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>同じ</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="9" t="n">
+    <row r="48" ht="36" customHeight="1">
+      <c r="A48" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>rename しない方式</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
         <is>
           <t>ある（fileName を書かない DirectWrite）</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D48" s="10" t="inlineStr">
         <is>
           <t>無い。必ず固定名 server.log に書き、回転時に rename</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E48" s="9" t="inlineStr">
         <is>
           <t>★違う</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="21" customHeight="1">
-      <c r="A31" s="5" t="n">
+    <row r="49" ht="21" customHeight="1">
+      <c r="A49" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>外から rename されたら開き直すか</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>しない</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>しない（SIGHUP 等で知らせる仕組みも無い）</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>同じ</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="21" customHeight="1">
-      <c r="A32" s="9" t="n">
+    <row r="50" ht="21" customHeight="1">
+      <c r="A50" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>以前の問題の「2人目の書き手」</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
         <is>
           <t>別タスク（別ホスト）</t>
         </is>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D50" s="10" t="inlineStr">
         <is>
           <t>同じタスク内の別 FD、または外部の rename</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t>★違う</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="21" customHeight="1">
-      <c r="A33" s="9" t="n">
+    <row r="51" ht="21" customHeight="1">
+      <c r="A51" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>タスクIDディレクトリの効果</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
         <is>
           <t>根治</t>
         </is>
       </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D51" s="10" t="inlineStr">
         <is>
           <t>効果なし</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr">
         <is>
           <t>★違う</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="9" t="n">
+    <row r="52" ht="36" customHeight="1">
+      <c r="A52" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>起きるタイミング</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
         <is>
           <t>デプロイと時境界が重なったとき（確率的）</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D52" s="10" t="inlineStr">
         <is>
           <t>犯人がいる限り毎日必ず（デプロイと無関係）</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>★違う</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="21" customHeight="1">
-      <c r="A35" s="9" t="n">
+    <row r="53" ht="21" customHeight="1">
+      <c r="A53" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>前日分のログ</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>シナリオD で消えることがある</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>原因候補1・3a・3b で毎日消える</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E53" s="9" t="inlineStr">
         <is>
           <t>★違う</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>※ 判別のヒント：デプロイしなかった日にも毎日起きているなら、ローリングアップデートとは無関係で、タスク内部（または外部 rename）に犯人がいることがほぼ確定します。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A43:E43"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A36:E36"/>
@@ -5078,7 +5405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5147,7 +5474,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="141" customHeight="1">
+    <row r="5" ht="156" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>1</t>
@@ -5162,7 +5489,7 @@
         <is>
           <t>・CLI で追加した別名ハンドラ（例 APP_FILE）の path が server.log
 ・logging-profile 内のハンドラ
-・WAR/EAR 同梱の logging.properties、jboss-logging.properties、log4j.xml（DailyRollingFileAppender）、log4j2.xml が ${jboss.server.log.dir}/server.log を指す（use-deployment-logging-config は既定 true）</t>
+・WAR/EAR の META-INF／WEB-INF/classes の logging.properties、jboss-logging.properties が ${jboss.server.log.dir}/server.log を指す（use-deployment-logging-config は既定 true。EAP 8.1 のコンテナが読むのはこの2つだけ）</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -5188,217 +5515,218 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>J1, J2</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="81" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+          <t>J1, J2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="141" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>アプリが同梱したログライブラリのアペンダ（EAP 8 で増えた経路）</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>・EAP 7 から移行したアプリが reload4j（log4j 1.x 互換）を WAR に同梱し、log4j.xml の DailyRollingFileAppender が ${jboss.server.log.dir}/server.log を指したまま
+・log4j-core／logback を同梱し API モジュールを除外している場合の log4j2.xml／logback.xml</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>EAP 8 はコンテナが log4j 1.x を提供しないので、log4j.xml はアプリ同梱の reload4j 自身が読み、自分で server.log を開いて rename する。use-deployment-logging-config では止まらない。reload4j は回転時に「移動先があれば先に削除 → rename」するため、JBoss が作った前日分を消し、JBoss が開いたばかりの新しい server.log を日付名にする。以後 JBoss の FILE は日付ファイルへ書き続ける。</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>完全一致（再現済み）</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>毎日消える</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>候補1と同じ（FD が2本以上）。audit-logging-config.sh が「有効（reload4j を同梱）」と判定</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>J2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="81" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>シェルのリダイレクト（JVM の stdout/stderr）</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>entrypoint で standalone.sh &gt;&gt; server.log 2&gt;&amp;1、| tee -a server.log</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>シェルが開いた FD を JVM が FD 1/2 として受け継ぎ、終了まで閉じない。CONSOLE ハンドラ・System.out の出力が、回転後は server.log.&lt;前日&gt; に書かれ続ける。FILE は新しい server.log に書く。</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>部分一致（server.log も伸びる）</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>残る</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>FD 1 / 2 が server.log* を指す</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>J3</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="66" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8" ht="66" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>3a</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>外部の rename（JBoss の回転の後）</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>コンテナ内の logrotate（dateext + dateformat .%Y-%m-%d で JBoss と同じ名前）、収集用 EC2 の cron、S3 退避バッチ、運用手順の mv</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>JBoss の回転で #1→日付名、新 #2。その後、外部が server.log(#2) を日付名へ mv（#1＝前日分を上書き削除）し、空の server.log(#3) を作る。JBoss は #2（名前は日付）へ1日中書く。</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>完全一致（再現済み）</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>消える</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>JVM の FD は1本だけなのに日付ファイルを指す。別ホストからの rename は名前表示が変わらないので inode で比較</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>J4</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="51" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="9" ht="51" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>3b</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>外部の rename（JBoss の回転の前）</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>同上で、実行が 0:00:00 直後</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>外部が #1→日付名、空の #2 を作る。JBoss の回転で #2（空）を日付名へ move（#1＝前日分を上書き削除）、新 #3 を open。</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>不一致（server.log に書かれる）</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>消える（日付ファイルが空）</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>日付ファイルが空／極端に小さい</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>J4</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="81" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="10" ht="81" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>タイムゾーンの不一致（見かけ上の類似）</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>コンテナの TZ が UTC のまま</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>「日付が変わった」判定が UTC の 0時＝JST 9時になる。JST 0〜9時のログは server.log に書かれ、9時に server.log.&lt;前日&gt; へ回転。後から見ると前日付ファイルに今日の 0〜9時のログがある。</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>見かけ上一致</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>残る</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>0〜9時の間に server.log が伸びているか。date と -Duser.timezone</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>J5</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>除外</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>rename の失敗</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>EFS の一時エラーなど</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>失敗すると JBoss は同じ server.log を開き直すので、ログは server.log に書かれ続ける。</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>逆の症状</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>残る</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>stderr の "Failed to move file"</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
@@ -5410,32 +5738,32 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>別タスク／front・back の共有</t>
+          <t>rename の失敗</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>EFS の一時エラーなど</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>タスクIDとコンテナ名でディレクトリを分離済み。</t>
+          <t>失敗すると JBoss は同じ server.log を開き直すので、ログは server.log に書かれ続ける。</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>該当しない</t>
+          <t>逆の症状</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>残る</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>念のため 19 シートの手順でパスを確認</t>
+          <t>stderr の "Failed to move file"</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -5452,162 +5780,216 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
+          <t>別タスク／front・back の共有</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>タスクIDとコンテナ名でディレクトリを分離済み。</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>該当しない</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>念のため 19 シートの手順でパスを確認</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>除外</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
           <t>EFS の性能・スループットモード</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>rename〜create の数ミリ秒が変わるだけで FD の行き先は変わらない。</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>該当しない</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>■ JBoss の回転処理の性質（jboss-logmanager 2.1.19.Final のソースで確認）</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>除外</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>起動時ログ（logging.properties）の FILE</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>subsystem の FILE と同名で引き継がれる同じハンドラ。FD は1本。</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>該当しない</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>J6（出力先をそろえる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>除外</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>EAP 8 のインストールマネージャ</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>standalone.sh の終了コード 20</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>JVM 終了後に順番に server.log へ書くだけで、同時には開かない。</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>該当しない</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>■ JBoss の回転処理の性質（EAP 8.1 と同じ jboss-logmanager 2.1.19.Final のソースで確認）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>性質</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>ソース上の根拠</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>今回への影響</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="51" customHeight="1">
-      <c r="A16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>回転はタイマーではなく次のログレコードで起きる</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>preWrite(): if (record.getMillis() &gt;= nextRollover) { rollOver(); ... }</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>ハンドラごとに別々に判定。0:00:00 ちょうどではなく「0時を過ぎて最初のログ」のとき</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="n"/>
-      <c r="H16" s="13" t="n"/>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>回転で閉じるのは自分の FD だけ</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>rollOver(): setFileInternal(null) → rotate → setFileInternal(file)</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>同じファイルを開いている別ハンドラ・別プロセスの FD は閉じない。そちらは日付ファイルに書き続ける</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
-      <c r="G17" s="12" t="n"/>
-      <c r="H17" s="13" t="n"/>
-    </row>
-    <row r="18" ht="51" customHeight="1">
-      <c r="A18" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>回転先は REPLACE_EXISTING（上書き）</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>SuffixRotator.move(): Files.move(src, target, StandardCopyOption.REPLACE_EXISTING)</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>2人目が回転すると、1人目が作った server.log.&lt;前日&gt;（前日分）を黙って消す</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="13" t="n"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr"/>
     </row>
     <row r="19" ht="51" customHeight="1">
       <c r="A19" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>開くのはいつも server.log</t>
+          <t>回転はタイマーではなく次のログレコードで起きる</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>FileHandler.setFile(): new FileOutputStream(file, append)（file は常に server.log）</t>
+          <t>preWrite(): if (record.getMillis() &gt;= nextRollover) { rollOver(); ... }</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>日付ファイルに書かれている＝古い FD が残っている、と断定できる</t>
+          <t>ハンドラごとに別々に判定。0:00:00 ちょうどではなく「0時を過ぎて最初のログ」のとき</t>
         </is>
       </c>
       <c r="E19" s="12" t="n"/>
@@ -5617,21 +5999,21 @@
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>外から rename されても開き直さない</t>
+          <t>回転で閉じるのは自分の FD だけ</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>開き直しは rollOver() の中だけ</t>
+          <t>rollOver(): setFileInternal(null) → rotate → setFileInternal(file)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>logrotate 等が rename すると、JBoss は日付ファイルに書き続ける</t>
+          <t>同じファイルを開いている別ハンドラ・別プロセスの FD は閉じない。そちらは日付ファイルに書き続ける</t>
         </is>
       </c>
       <c r="E20" s="12" t="n"/>
@@ -5641,21 +6023,21 @@
     </row>
     <row r="21" ht="51" customHeight="1">
       <c r="A21" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>日付の切り替わりは JVM（ハンドラ）のタイムゾーン</t>
+          <t>回転先は REPLACE_EXISTING（上書き）</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>calcNextRollover(): Calendar.getInstance(timeZone)（既定は JVM 既定）</t>
+          <t>SuffixRotator.move(): Files.move(src, target, StandardCopyOption.REPLACE_EXISTING)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>UTC のままだと回転は JST 09:00</t>
+          <t>2人目が回転すると、1人目が作った server.log.&lt;前日&gt;（前日分）を黙って消す</t>
         </is>
       </c>
       <c r="E21" s="12" t="n"/>
@@ -5665,21 +6047,21 @@
     </row>
     <row r="22" ht="51" customHeight="1">
       <c r="A22" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>rename 失敗時は同じ server.log を開き直す</t>
+          <t>開くのはいつも server.log</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>move() は例外を ErrorManager に出すだけで、続けて setFileInternal(file)</t>
+          <t>FileHandler.setFile(): new FileOutputStream(file, append)（file は常に server.log）</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>「rename 失敗」は今回と逆の症状。原因ではない</t>
+          <t>日付ファイルに書かれている＝古い FD が残っている、と断定できる</t>
         </is>
       </c>
       <c r="E22" s="12" t="n"/>
@@ -5687,18 +6069,90 @@
       <c r="G22" s="12" t="n"/>
       <c r="H22" s="13" t="n"/>
     </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>外から rename されても開き直さない</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>開き直しは rollOver() の中だけ</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>logrotate 等が rename すると、JBoss は日付ファイルに書き続ける</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="51" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>日付の切り替わりは JVM（ハンドラ）のタイムゾーン</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>calcNextRollover(): Calendar.getInstance(timeZone)（既定は JVM 既定）</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>UTC のままだと回転は JST 09:00</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="13" t="n"/>
+    </row>
+    <row r="25" ht="51" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>rename 失敗時は同じ server.log を開き直す</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>move() は例外を ErrorManager に出すだけで、続けて setFileInternal(file)</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>「rename 失敗」は今回と逆の症状。原因ではない</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="13" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="D21:H21"/>
+    <mergeCell ref="D25:H25"/>
     <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D16:H16"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="D19:H19"/>
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="D23:H23"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5728,10 +6182,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>#1, #2, #3 は inode 番号。同じロガーに FILE → APP_FILE の順でハンドラが付いている場合。どちらが先に回転しても症状の形は同じ。</t>
+          <t>#1, #2, #3 は inode 番号。同じロガーに FILE → APP_FILE の順でハンドラが付いている場合。どちらが先に回転しても症状の形は同じ。原因候補1b（APP_FILE の代わりにアプリ同梱 reload4j の DailyRollingFileAppender）も同じ流れ。reload4j は rename の前に既存の日付ファイルを delete する点だけが違う。</t>
         </is>
       </c>
     </row>
@@ -6346,7 +6800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6359,14 +6813,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>実物の jboss-logmanager での再現結果（2026-09-24 実行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
+          <t>EAP 8.1 と同じライブラリでの再現結果（2026-09-24 実行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="43" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>jboss/repro/ServerLogRotationRepro.java を jboss-logmanager 2.1.19.Final（EAP 7.4 系と同じ系列）で実行。JBoss 本体は不要。ログの時刻を 9/18 23:59 → 9/19 0:00 に設定して日付またぎを起こす。全文は jboss/repro/expected_output.txt。</t>
+          <t>jboss/repro/ServerLogRotationRepro.java を EAP 8.1 と同じ jboss-logmanager 2.1.19.Final ＋ wildfly-common 1.7.0.Final（JDK 21）で実行。JBoss 本体は不要。S6 は MixedLibraryRepro.java（JBoss FILE ＋ 同梱 reload4j 1.2.26）を実時計で分の境界をまたいで実行。ログの時刻を 9/18 23:59 → 9/19 0:00 に設定して日付またぎを起こす。全文は jboss/repro/expected_output.txt。</t>
         </is>
       </c>
     </row>
@@ -6589,29 +7043,57 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>S6 JBoss FILE ＋ 同梱 reload4j（原因候補1b）</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>fd 10 → server.log.&lt;前の期間&gt;（JBoss）
+fd 11 → server.log（reload4j）</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>reload4j の行だけ</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>JBoss FILE の境界後の行（境界前の行は reload4j の target.delete() で消滅）</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>症状と一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>★ S1・S2 とも、ハンドラ自身は getFile()=server.log を返す（「server.log に書いているつもり」）。管理 CLI でハンドラ設定を見ても異常は見えず、FD を見て初めて分かる。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>■ S1 の実際の出力（抜粋）</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="51" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="51" t="inlineStr">
         <is>
           <t>▼ S1 の出力</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="195.5" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17" ht="195.5" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  ■ この JVM が開いている FD（/proc/self/fd）
     fd 8 -&gt; server.log.2026-09-18
@@ -6629,69 +7111,114 @@
         FILE     | 2026-09-19 12:00:00 9/19 昼のログ</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="13" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="13" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>■ S6（JBoss FILE ＋ 同梱 reload4j）の実際の出力（抜粋）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="51" t="inlineStr">
+        <is>
+          <t>▼ S6 の出力</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="233" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ■ この JVM が開いている FD（/proc/self/fd）
+    fd 10 -&gt; server.log.2026-09-24-06-49
+    fd 11 -&gt; server.log
+    ※ JBoss の FILE も reload4j も「server.log に書いているつもり」
+  ■ ディレクトリの状態と中身
+    server.log  (181 bytes)
+        RELOAD4J | 06:50:00 ログ 6 件目
+        RELOAD4J | 06:50:01 ログ 7 件目
+        RELOAD4J | 06:50:02 ログ 8 件目
+        RELOAD4J | 06:50:03 ログ 9 件目
+        RELOAD4J | 06:50:04 ログ 10 件目
+    server.log.2026-09-24-06-49  (181 bytes)
+        FILE     | 06:50:00 ログ 6 件目
+        FILE     | 06:50:01 ログ 7 件目
+        FILE     | 06:50:02 ログ 8 件目
+        FILE     | 06:50:03 ログ 9 件目
+        FILE     | 06:50:04 ログ 10 件目</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="13" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>■ 自分の環境で再現する</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="51" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="51" t="inlineStr">
         <is>
           <t>▼ 手元で再現</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="45.5" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>cd jboss/repro
 ./run_repro.sh                         # jar を Maven Central から取得して実行（Java 17 以上）
-LOGMANAGER_VERSION=2.1.18.Final ./run_repro.sh   # 実環境の EAP に合わせてバージョンを変える</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="13" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="51" t="inlineStr">
+./run_repro.sh --reload4j              # 原因候補1b（JBoss FILE ＋ 同梱 reload4j）。最大 70 秒
+LOGMANAGER_VERSION=&lt;実機の版&gt; ./run_repro.sh      # 実機の modules の jar 名に合わせる（既定は EAP 8.1 と同じ 2.1.19.Final）</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="13" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="51" t="inlineStr">
         <is>
           <t>▼ EFS 上で再現</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20.5" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="27" ht="20.5" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>./run_repro.sh /mnt/efs/logs/repro    # 出力先を EFS にすれば、EFS 上で同じ結果になることを確認できる</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="13" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="13" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="14">
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6704,7 +7231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6800,15 +7327,15 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="51" customHeight="1">
+    <row r="7" ht="66" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J2a</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>デプロイメント内のログ設定を無効化（use-deployment-logging-config=false）、またはアプリ側の出力先を server.log 以外へ変更</t>
+          <t>コンテナが読むデプロイメント内ログ設定を無効化（use-deployment-logging-config=false。対象は logging.properties／jboss-logging.properties だけ）</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -6832,20 +7359,20 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="51" customHeight="1">
+    <row r="8" ht="81" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J2b</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>entrypoint で stdout/stderr を server.log にリダイレクトしない（stdout は ECS の awslogs / FireLens へ）</t>
+          <t>アプリ同梱ライブラリ（reload4j の log4j.xml、log4j-core の log4j2.xml、logback の logback.xml）の出力先を server.log 以外へ変更。アプリ用ファイルは第9章の案2（DirectWrite＋タスクID別パス）で書く</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>候補2</t>
+          <t>候補1b</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -6855,234 +7382,248 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>極小</t>
+          <t>小（アプリ改修）</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>jboss/bin/entrypoint.sh</t>
+          <t>アプリの設定ファイル</t>
         </is>
       </c>
     </row>
     <row r="9" ht="51" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>entrypoint で stdout/stderr を server.log にリダイレクトしない（stdout は ECS の awslogs / FireLens へ）</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>候補2</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>根治</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>極小</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>jboss/bin/entrypoint.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="51" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
           <t>J4</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>logrotate・収集バッチ・運用手順に server.log を触らせない（触ってよいのは回転済みの server.log.* で、1日以上前のものだけ）</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>候補3</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>根治</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>小</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>運用手順・cron の修正</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>J5</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>TZ=Asia/Tokyo と -Duser.timezone=Asia/Tokyo を設定</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>候補4</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>誤認防止</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>極小</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>jboss/bin/entrypoint.sh</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="51" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="12" ht="51" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>J6</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>JBOSS_LOG_DIR と -Djboss.server.log.dir を同じにする（起動時ログと本番ログの出力先をそろえる）</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>予防</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>予防</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>極小</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>jboss/bin/entrypoint.sh</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>J7</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>監視：check-server-log-fd.sh を日次（0:05 など）で実行し、終了コード 1 でアラート</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>全部</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>検知</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>小</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>jboss/bin/check-server-log-fd.sh</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="66" customHeight="1">
-      <c r="A13" s="42" t="inlineStr">
+    <row r="14" ht="66" customHeight="1">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>J8</t>
         </is>
       </c>
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t>【恒久策】server.log をやめ、JSON で stdout に出す（CONSOLE + json-formatter。EAP 7.1 以降）</t>
-        </is>
-      </c>
-      <c r="C13" s="42" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>【恒久策】server.log をやめ、JSON で stdout に出す（CONSOLE + json-formatter。EAP 8.1 の管理モデルに json-formatter・zone-id があることをソースで確認済み）</t>
+        </is>
+      </c>
+      <c r="C14" s="42" t="inlineStr">
         <is>
           <t>全部</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
+      <c r="D14" s="42" t="inlineStr">
         <is>
           <t>根治（ファイルも rename も無くなる）</t>
         </is>
       </c>
-      <c r="E13" s="42" t="inlineStr">
+      <c r="E14" s="42" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F13" s="44" t="inlineStr">
+      <c r="F14" s="44" t="inlineStr">
         <is>
           <t>jboss/cli/server-log-to-stdout.cli</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>推奨の組み合わせ：まず J7（診断）で犯人を特定 → 候補1なら J1＋J2／候補2なら J3／候補3なら J4 → 併用で J5・J6 → 恒久策として J8（アプリログの案1とそろえると収集経路が1本になる）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>推奨の組み合わせ：まず J7（診断）で犯人を特定 → 候補1なら J1＋J2a／候補1b なら J2b／候補2なら J3／候補3なら J4 → 併用で J5・J6 → 恒久策として J8（アプリログの案1とそろえると収集経路が1本になる）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>■ やっても効かないこと</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>対策</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>効かない理由</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>タスクIDディレクトリをさらに細かくする</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>犯人は同じディレクトリの中にいる（14 シート）</t>
         </is>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>autoflush を変える</t>
+          <t>タスクIDディレクトリをさらに細かくする</t>
         </is>
       </c>
       <c r="C19" s="12" t="n"/>
@@ -7090,17 +7631,17 @@
       <c r="E19" s="13" t="n"/>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>書き込むタイミングが変わるだけで、FD の行き先は変わらない</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1">
+          <t>犯人は同じディレクトリの中にいる（14 シート）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="51" customHeight="1">
       <c r="A20" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>size-rotating / periodic-size-rotating に替える</t>
+          <t>use-deployment-logging-config=false だけで済ませる</t>
         </is>
       </c>
       <c r="C20" s="12" t="n"/>
@@ -7108,17 +7649,17 @@
       <c r="E20" s="13" t="n"/>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>回転の方式（close → rename → create）は同じ。2人目がいれば同じことが起きる</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="66" customHeight="1">
+          <t>EAP 8.1 でこれが止めるのは logging.properties／jboss-logging.properties だけ。アプリ同梱の reload4j 等（候補1b）は止まらない</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="51" customHeight="1">
       <c r="A21" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>suffix に .gz を付ける</t>
+          <t>jboss-deployment-structure.xml で logging サブシステムを除外する</t>
         </is>
       </c>
       <c r="C21" s="12" t="n"/>
@@ -7126,17 +7667,17 @@
       <c r="E21" s="13" t="n"/>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>回転時に圧縮して元ファイルを削除するので、2人目の FD は削除済みファイル（EFS では .nfs*）を指し、ログがどこにも残らなくなる。悪化する</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="21" customHeight="1">
+          <t>アプリ同梱ライブラリが自分でファイルを開くことは変わらない。むしろ候補1b が有効になる条件になる</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>async-handler で FILE を包む</t>
+          <t>autoflush を変える</t>
         </is>
       </c>
       <c r="C22" s="12" t="n"/>
@@ -7144,17 +7685,17 @@
       <c r="E22" s="13" t="n"/>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>非同期になるだけで、FD の本数は変わらない</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="21" customHeight="1">
+          <t>書き込むタイミングが変わるだけで、FD の行き先は変わらない</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>JBoss の再起動</t>
+          <t>size-rotating / periodic-size-rotating に替える</t>
         </is>
       </c>
       <c r="C23" s="12" t="n"/>
@@ -7162,98 +7703,98 @@
       <c r="E23" s="13" t="n"/>
       <c r="F23" s="6" t="inlineStr">
         <is>
+          <t>回転の方式（close → rename → create）は同じ。2人目がいれば同じことが起きる</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="66" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>suffix に .gz を付ける</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>回転時に圧縮して元ファイルを削除するので、2人目の FD は削除済みファイル（EFS では .nfs*）を指し、ログがどこにも残らなくなる。悪化する</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="21" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>async-handler で FILE を包む</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>非同期になるだけで、FD の本数は変わらない</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="21" customHeight="1">
+      <c r="A26" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>JBoss の再起動</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
           <t>一時的に直るが、翌日 0時にまた起きる</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>■ 実装ファイル（リポジトリ jboss/ 配下）</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>ファイル</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>役割</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="31" customHeight="1">
-      <c r="A27" s="5" t="n">
+    <row r="30" ht="31" customHeight="1">
+      <c r="A30" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>jboss/repro/ServerLogRotationRepro.java</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>実物の jboss-logmanager で原因候補1〜4を再現し、FD と各ファイルの中身を表示</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="31" customHeight="1">
-      <c r="A28" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>jboss/repro/run_repro.sh</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>必要な jar を取得して実行。引数に EFS 上のパスを渡せば EFS 上で再現</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>jboss/repro/expected_output.txt</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-24 の実行結果（17 シートの根拠）</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="56" customHeight="1">
-      <c r="A30" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>jboss/bin/check-server-log-fd.sh</t>
         </is>
       </c>
       <c r="C30" s="12" t="n"/>
@@ -7261,17 +7802,17 @@
       <c r="E30" s="13" t="n"/>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>実行時診断。/proc/*/fd から server.log* を指す FD の本数・番号・inode を調べて原因候補を自動判定（終了コード 0=正常 / 1=異常）</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="68.5" customHeight="1">
+          <t>実物の jboss-logmanager で原因候補1〜4を再現し、FD と各ファイルの中身を表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="31" customHeight="1">
       <c r="A31" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>jboss/bin/audit-logging-config.sh</t>
+          <t>jboss/repro/run_repro.sh</t>
         </is>
       </c>
       <c r="C31" s="12" t="n"/>
@@ -7279,17 +7820,17 @@
       <c r="E31" s="13" t="n"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>静的点検。standalone.xml（logging-profile 含む）・logging.properties・デプロイメント内ログ設定・logrotate/cron・entrypoint を横断して「server.log を開く／rename する主体」を列挙</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="43.5" customHeight="1">
+          <t>必要な jar を取得して実行。引数に EFS 上のパスを渡せば EFS 上で再現</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="31" customHeight="1">
       <c r="A32" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>jboss/cli/fix-server-log-single-writer.cli</t>
+          <t>jboss/repro/expected_output.txt</t>
         </is>
       </c>
       <c r="C32" s="12" t="n"/>
@@ -7297,17 +7838,17 @@
       <c r="E32" s="13" t="n"/>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>J1・J2：FILE を唯一の server.log ハンドラにし、2つ目を別ファイルへ向け直し、デプロイメント内ログ設定を無効化</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="31" customHeight="1">
+          <t>2026-09-24 に EAP 8.1 と同じライブラリで実行した結果（17 シートの根拠）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="43.5" customHeight="1">
       <c r="A33" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>jboss/cli/server-log-to-stdout.cli</t>
+          <t>jboss/repro/MixedLibraryRepro.java</t>
         </is>
       </c>
       <c r="C33" s="12" t="n"/>
@@ -7315,17 +7856,17 @@
       <c r="E33" s="13" t="n"/>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>J8：server.log をやめて JSON で stdout に出す</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="43.5" customHeight="1">
+          <t>原因候補1b：JBoss FILE とアプリ同梱 reload4j が同じ server.log を回転させる様子を実時計で再現（run_repro.sh --reload4j）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
       <c r="A34" s="5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>jboss/bin/entrypoint.sh</t>
+          <t>jboss/repro/expected_output_reload4j.txt</t>
         </is>
       </c>
       <c r="C34" s="12" t="n"/>
@@ -7333,26 +7874,116 @@
       <c r="E34" s="13" t="n"/>
       <c r="F34" s="6" t="inlineStr">
         <is>
+          <t>上記の実行結果</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="56" customHeight="1">
+      <c r="A35" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>jboss/bin/check-server-log-fd.sh</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>実行時診断。/proc/*/fd から server.log* を指す FD の本数・番号・inode を調べて原因候補を自動判定（終了コード 0=正常 / 1=異常）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="118.5" customHeight="1">
+      <c r="A36" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>jboss/bin/audit-logging-config.sh</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n"/>
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>静的点検。standalone.xml（logging-profile 含む）・logging.properties・デプロイメント内ログ設定・logrotate/cron・entrypoint を横断して「server.log を開く／rename する主体」を列挙。デプロイメント内設定は EAP 8.1 の仕様で「コンテナが読む／同梱 reload4j・log4j-core・logback が読む／無視」に分類し、同梱 jar と除外設定から実際に有効かを判定</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="43.5" customHeight="1">
+      <c r="A37" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>jboss/cli/fix-server-log-single-writer.cli</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="12" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>J1・J2a：FILE を唯一の server.log ハンドラにし、2つ目を別ファイルへ向け直し、デプロイメント内ログ設定を無効化</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="31" customHeight="1">
+      <c r="A38" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>jboss/cli/server-log-to-stdout.cli</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>J8：server.log をやめて JSON で stdout に出す</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="43.5" customHeight="1">
+      <c r="A39" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>jboss/bin/entrypoint.sh</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="13" t="n"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
           <t>J3・J5・J6：タスクID／コンテナ名のディレクトリを作り、リダイレクトせずに exec standalone.sh</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>■ 設定例（そのままコピーできます）</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="51" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="51" t="inlineStr">
         <is>
           <t>▼ jboss/bin/entrypoint.sh</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="383" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="43" ht="383" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>#!/bin/sh
 # entrypoint.sh（JBoss EAP コンテナ用）
@@ -7383,21 +8014,21 @@
 #   standalone.sh は JBOSS_LOG_DIR から起動時ログ（-Dorg.jboss.boot.log.file）の場所を決め、</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="12" t="n"/>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="13" t="n"/>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="51" t="inlineStr">
+      <c r="B43" s="12" t="n"/>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="13" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="51" t="inlineStr">
         <is>
           <t>▼ jboss/bin/entrypoint.sh（続き 2/2）</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="245.5" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
+    <row r="45" ht="245.5" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>#   -Djboss.server.log.dir から subsystem の FILE ハンドラの場所を決める。
 #   2つを必ず同じディレクトリにする（食い違うと起動直後だけ別の server.log に書かれる）。
@@ -7418,21 +8049,21 @@
   "$@"</t>
         </is>
       </c>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12" t="n"/>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="13" t="n"/>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="51" t="inlineStr">
+      <c r="B45" s="12" t="n"/>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="13" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="51" t="inlineStr">
         <is>
           <t>▼ jboss/cli/fix-server-log-single-writer.cli</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="383" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="47" ht="383" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t># fix-server-log-single-writer.cli
 #   server.log を「開く」のも「rename する」のも FILE ハンドラ1つだけにする。
@@ -7463,21 +8094,21 @@
 # ---------------------------------------------------------------------------------------------</t>
         </is>
       </c>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12" t="n"/>
-      <c r="E42" s="12" t="n"/>
-      <c r="F42" s="13" t="n"/>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="51" t="inlineStr">
+      <c r="B47" s="12" t="n"/>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="12" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="13" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="51" t="inlineStr">
         <is>
           <t>▼ jboss/cli/fix-server-log-single-writer.cli（続き 2/2）</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="270.5" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+    <row r="49" ht="358" customHeight="1">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>if (outcome == success) of /subsystem=logging/periodic-rotating-file-handler=APP_FILE:read-resource
     /subsystem=logging/periodic-rotating-file-handler=APP_FILE:write-attribute(name=file, value={relative-to=jboss.server.log.dir, path=app.log})
@@ -7487,37 +8118,44 @@
     /subsystem=logging/logging-profile=app/periodic-rotating-file-handler=FILE:write-attribute(name=file, value={relative-to=jboss.server.log.dir, path=app-profile.log})
 end-if
 # ---------------------------------------------------------------------------------------------
-# 3) デプロイメント（WAR/EAR）に同梱された logging.properties / log4j.xml / log4j2.xml 等を無視させる
-#    これらが ${jboss.server.log.dir}/server.log を指していると、JBoss の FILE とは別の FD で
-#    server.log を開き、しかも独自に rename する（log4j 1.x DailyRollingFileAppender の既定サフィックスは
-#    '.'yyyy-MM-dd なので、JBoss と全く同じ server.log.YYYY-MM-DD という名前になる）。
-#    ★ アプリが自前のログ設定に依存している場合は、この設定ではなく、アプリ側の出力先を
-#      server.log 以外（app.log 等）へ変える方を選んでください。
+# 3) デプロイメント（WAR/EAR）の META-INF / WEB-INF/classes にある logging.properties・
+#    jboss-logging.properties をコンテナに読ませない（EAP 8.1 でコンテナが読むのはこの2つだけ）。
+#    これらが ${jboss.server.log.dir}/server.log を指していると、デプロイメント専用の LogContext に
+#    JBoss の FILE とは別の PeriodicRotatingFileHandler が作られ、別の FD で server.log を開いて独自に rename する。
+#
+#    ★ この設定では止まらないもの（アプリ側の修正が必要）：
+#      - WAR に reload4j / log4j 1.2 を同梱し、log4j.xml / log4j.properties で server.log を指している
+#        （EAP 8 はコンテナが log4j 1.x を提供しないため、アプリのライブラリ自身が設定を読み、
+#         DailyRollingFileAppender が server.log を開いて rename する。既定の日付パターン '.'yyyy-MM-dd は
+#         JBoss と全く同じ server.log.YYYY-MM-DD という名前になる）
+#      - log4j-core / logback を同梱し、コンテナのログ API モジュールを除外している場合の log4j2.xml / logback.xml
+#      → いずれもアプリ側の出力先を server.log 以外（app.log 等）に変えること。audit-logging-config.sh が判定する。
+#    ★ アプリが logging.properties に依存している場合も、この設定ではなく出力先の変更を選ぶ。
 # ---------------------------------------------------------------------------------------------
 /subsystem=logging:write-attribute(name=use-deployment-logging-config, value=false)
 stop-embedded-server</t>
         </is>
       </c>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="12" t="n"/>
-      <c r="F44" s="13" t="n"/>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="51" t="inlineStr">
+      <c r="B49" s="12" t="n"/>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="13" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="51" t="inlineStr">
         <is>
           <t>▼ jboss/cli/server-log-to-stdout.cli</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="295.5" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+    <row r="51" ht="295.5" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t># server-log-to-stdout.cli
 #   【恒久対策】server.log というファイル自体をやめ、JSON で stdout に出す。
 #   stdout は ECS の awslogs / FireLens(Fluent Bit) が拾うので、ファイルも FD も rename も存在しなくなる。
-#   （本資料 9.1 の「案1」を JBoss に適用したもの。EAP 7.1 以降の json-formatter を使用）
+#   （本資料 9.1 の「案1」を JBoss に適用したもの。json-formatter の zone-id 等は EAP 8.1＝WildFly Core 27 のソースで確認済み）
 #
 #     $JBOSS_HOME/bin/jboss-cli.sh --file=server-log-to-stdout.cli
 embed-server --server-config=standalone.xml --std-out=discard
@@ -7535,53 +8173,57 @@
 stop-embedded-server</t>
         </is>
       </c>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-      <c r="F46" s="13" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>※ use-deployment-logging-config=false にすると、アプリ同梱のログ設定はすべて無視されます。アプリがそれに依存している場合は、アプリ側の出力先を server.log 以外に変え、そのファイルは第9章の案2（DirectWrite ＋ タスクID別パス）で書いてください。</t>
+      <c r="B51" s="12" t="n"/>
+      <c r="C51" s="12" t="n"/>
+      <c r="D51" s="12" t="n"/>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="13" t="n"/>
+    </row>
+    <row r="52" ht="43" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>※ use-deployment-logging-config=false にすると、コンテナが読む logging.properties／jboss-logging.properties が無視されます（EAP 8.1）。アプリがそれに依存している場合や、reload4j 等を同梱している場合（候補1b）は、アプリ側の出力先を server.log 以外に変え、そのファイルは第9章の案2（DirectWrite ＋ タスクID別パス）で書いてください。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="36">
     <mergeCell ref="A41:F41"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="A50:F50"/>
     <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B36:E36"/>
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B26:E26"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="A43:F43"/>
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="B21:E21"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A15:F15"/>
     <mergeCell ref="B23:E23"/>
-    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A51:F51"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A45:F45"/>
-    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B38:E38"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8397,7 +9039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8808,200 +9450,200 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>WAR/EAR に logging.properties・jboss-logging.properties・log4j.xml・log4j2.xml が同梱されていないか／server.log を指していないか</t>
+          <t>WAR/EAR の META-INF／WEB-INF/classes に logging.properties・jboss-logging.properties がないか／server.log を指していないか</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>audit-logging-config.sh の 3</t>
+          <t>audit-logging-config.sh の 3 (a)</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
       <c r="F25" s="6" t="inlineStr"/>
     </row>
-    <row r="26" ht="36" customHeight="1">
+    <row r="26" ht="66" customHeight="1">
       <c r="A26" s="5" t="n">
         <v>8</v>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>候補3</t>
+          <t>候補1b</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>コンテナ内の /etc/logrotate.d・cron、収集用 EC2 の cron、運用手順に server.log の rename が無いか</t>
+          <t>WAR/EAR に reload4j／log4j 1.2 の jar が同梱されていないか。同梱されていれば log4j.xml／log4j.properties の出力先が server.log でないか（EAP 7 から移行したアプリは特に注意）</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>audit-logging-config.sh の 4 ＋ 目視</t>
+          <t>audit-logging-config.sh の 3 (b)</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
       <c r="F26" s="6" t="inlineStr"/>
     </row>
-    <row r="27" ht="21" customHeight="1">
+    <row r="27" ht="66" customHeight="1">
       <c r="A27" s="5" t="n">
         <v>9</v>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>候補2</t>
+          <t>候補1b</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>entrypoint に &gt;&gt; server.log や | tee が無いか</t>
+          <t>log4j-core／logback を同梱し、jboss-deployment-structure.xml でコンテナのログ API モジュールを除外していないか。していれば log4j2.xml／logback.xml の出力先を確認</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>audit-logging-config.sh の 5</t>
+          <t>audit-logging-config.sh の 3 (c)(d)</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr"/>
       <c r="F27" s="6" t="inlineStr"/>
     </row>
-    <row r="28" ht="21" customHeight="1">
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="5" t="n">
         <v>10</v>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>候補4</t>
+          <t>候補3</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>コンテナの date と JVM の user.timezone が JST か</t>
+          <t>コンテナ内の /etc/logrotate.d・cron、収集用 EC2 の cron、運用手順に server.log の rename が無いか</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>上の #6</t>
+          <t>audit-logging-config.sh の 4 ＋ 目視</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr"/>
       <c r="F28" s="6" t="inlineStr"/>
     </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="29" ht="21" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>候補2</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>entrypoint に &gt;&gt; server.log や | tee が無いか</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>audit-logging-config.sh の 5</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30" ht="21" customHeight="1">
+      <c r="A30" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>候補4</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>コンテナの date と JVM の user.timezone が JST か</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>上の #6</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>■ チェックリスト：対策の実施</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>区分</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>実施項目</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>参照</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>状態</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>結果・メモ</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="21" customHeight="1">
-      <c r="A32" s="5" t="n">
+    <row r="34" ht="21" customHeight="1">
+      <c r="A34" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>対策</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>犯人に応じて J1〜J4 を実施</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>犯人に応じて J1・J2a・J2b・J3・J4 を実施</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>18 シート</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="21" customHeight="1">
-      <c r="A33" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>対策</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>J5（TZ）と J6（ログディレクトリの一致）を実施</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>18 シート</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr"/>
-      <c r="F33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>検証</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>ステージングで 0時をまたいで稼働させ、check-server-log-fd.sh が「正常」になることを確認</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>上の #1</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
       <c r="F34" s="6" t="inlineStr"/>
     </row>
-    <row r="35" ht="36" customHeight="1">
+    <row r="35" ht="21" customHeight="1">
       <c r="A35" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>監視</t>
+          <t>対策</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>本番適用後、check-server-log-fd.sh を日次監視に組み込む（J7）</t>
+          <t>J5（TZ）と J6（ログディレクトリの一致）を実施</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -9014,168 +9656,250 @@
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>恒久</t>
+          <t>検証</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>恒久策 J8（stdout ＋ FireLens／awslogs）の採否を、アプリログの案1とあわせて決める</t>
+          <t>ステージングで 0時をまたいで稼働させ、check-server-log-fd.sh が「正常」になることを確認</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>07・08・18 シート</t>
+          <t>上の #1</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
       <c r="F36" s="6" t="inlineStr"/>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>監視</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>本番適用後、check-server-log-fd.sh を日次監視に組み込む（J7）</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>18 シート</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>恒久</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>恒久策 J8（stdout ＋ FireLens／awslogs）の採否を、アプリログの案1とあわせて決める</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>07・08・18 シート</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>■ 要確認事項</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40" ht="96" customHeight="1">
-      <c r="A40" s="5" t="n">
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="126" customHeight="1">
+      <c r="A42" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>jboss-logmanager のバージョン</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>本シート群は EAP 7.4 系と同じ 2.1 系（2.1.19.Final）のソースと実行結果に基づく。EAP 7.0〜7.3（2.0 系）・EAP 8（3.x 系）も回転手順（close → move → open）は同じ設計だが、run_repro.sh の LOGMANAGER_VERSION を実環境に合わせて確認する。EAP 6 系（1.5 系）は File.renameTo だが、Linux では移動先を上書きする点は同じ。</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="13" t="n"/>
-    </row>
-    <row r="41" ht="51" customHeight="1">
-      <c r="A41" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>ハンドラの呼び出し順</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>同じロガーに複数ハンドラがある場合は登録順。どちらが日付ファイルに書き続けるかは順序で変わるが、症状の形は変わらない。</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="n"/>
-      <c r="F41" s="13" t="n"/>
-    </row>
-    <row r="42" ht="51" customHeight="1">
-      <c r="A42" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>実行時リソース</t>
-        </is>
-      </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>audit-logging-config.sh --cli の /deployment=*/subsystem=logging/configuration=* は EAP 7 系の実行時リソース。EAP 6 系では静的点検で代替する。</t>
+          <t>本シート群は EAP 8.1 と同じ 2.1.19.Final（EAP 8.1 → WildFly 35 → WildFly Core 27 の上流 POM で特定）のソースと実行結果に基づく。Red Hat の製品リポジトリ・カスタマーポータルは検証環境から参照できなかったため、実機の $JBOSS_HOME/modules/system/layers/base/org/jboss/logmanager/main/ の jar 名で最終確認する。累積パッチで差し替わっていれば LOGMANAGER_VERSION=&lt;版&gt; ./run_repro.sh で再確認できる。</t>
         </is>
       </c>
       <c r="D42" s="12" t="n"/>
       <c r="E42" s="12" t="n"/>
       <c r="F42" s="13" t="n"/>
     </row>
-    <row r="43" ht="36" customHeight="1">
+    <row r="43" ht="51" customHeight="1">
       <c r="A43" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>別ホストからの rename</t>
+          <t>ハンドラの呼び出し順</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>/proc/&lt;pid&gt;/fd の表示名が更新されるかは NFS クライアントのキャッシュ次第。inode 番号での比較を正とする。</t>
+          <t>同じロガーに複数ハンドラがある場合は登録順。どちらが日付ファイルに書き続けるかは順序で変わるが、症状の形は変わらない。</t>
         </is>
       </c>
       <c r="D43" s="12" t="n"/>
       <c r="E43" s="12" t="n"/>
       <c r="F43" s="13" t="n"/>
     </row>
-    <row r="44" ht="66" customHeight="1">
+    <row r="44" ht="96" customHeight="1">
       <c r="A44" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>コンテナ間の PID 名前空間</t>
+          <t>実行時リソース</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>タスク定義で pidMode: task でない場合、サイドカーが server.log を開いていても JBoss コンテナからは見えない。サイドカーの中でも check-server-log-fd.sh を実行する。</t>
+          <t>audit-logging-config.sh --cli の /deployment=*/subsystem=logging/configuration=* は WildFly Core 27 のソースで EAP 8.1 に存在することを確認済み。ただし見えるのは候補1（コンテナが読む logging.properties）だけで、候補1b（同梱 reload4j 等）は管理モデルに現れない。静的点検と FD 点検で確認する。</t>
         </is>
       </c>
       <c r="D44" s="12" t="n"/>
       <c r="E44" s="12" t="n"/>
       <c r="F44" s="13" t="n"/>
     </row>
+    <row r="45" ht="66" customHeight="1">
+      <c r="A45" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>EAP 8.1 のコンテナイメージ</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Red Hat 提供の EAP 8.1 イメージを使っている場合は、起動スクリプトが標準出力をどう扱うかを確認（audit-logging-config.sh &lt;起動スクリプト&gt; で点検）。ZIP 版から自作したイメージなら entrypoint.sh の方式でよい。</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="13" t="n"/>
+    </row>
+    <row r="46" ht="66" customHeight="1">
+      <c r="A46" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>EAR の除外設定</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>jboss-deployment-structure.xml の除外が &lt;deployment&gt; と &lt;sub-deployment&gt; のどちらにあるかで効く範囲が変わる。audit-logging-config.sh はどちらかにあれば有効の可能性ありと判定するので、該当したら目で確認する。</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="13" t="n"/>
+    </row>
+    <row r="47" ht="36" customHeight="1">
+      <c r="A47" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>別ホストからの rename</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>/proc/&lt;pid&gt;/fd の表示名が更新されるかは NFS クライアントのキャッシュ次第。inode 番号での比較を正とする。</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="13" t="n"/>
+    </row>
+    <row r="48" ht="66" customHeight="1">
+      <c r="A48" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>コンテナ間の PID 名前空間</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>タスク定義で pidMode: task でない場合、サイドカーが server.log を開いていても JBoss コンテナからは見えない。サイドカーの中でも check-server-log-fd.sh を実行する。</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="n"/>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="13" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="D11:F11"/>
+    <mergeCell ref="C48:F48"/>
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="C42:F42"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="C45:F45"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="C41:F41"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="C47:F47"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="C44:F44"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="C40:F40"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C43:F43"/>
+    <mergeCell ref="C46:F46"/>
     <mergeCell ref="D6:F6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E19:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E19:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未着手,実施中,完了,該当なし"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>